<commit_message>
feat(frontend): tornar gráficos configuráveis com Recharts e validar backend/frontend
</commit_message>
<xml_diff>
--- a/relatorio_olimpo/relatorio_olimpo_ic.xlsx
+++ b/relatorio_olimpo/relatorio_olimpo_ic.xlsx
@@ -423,10 +423,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
           <t>polimento automotivo</t>
@@ -455,1042 +460,1062 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>45781</v>
+        <v>45809</v>
       </c>
       <c r="B2" t="n">
-        <v>71.49014245903369</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>52.29231199877616</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>59.51614286500197</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>51.32887255572378</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>27.06019074522419</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>45788</v>
+        <v>45816</v>
       </c>
       <c r="B3" t="n">
-        <v>71.42853145645715</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>58.03494044948112</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>62.44103547709076</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>44.36916460455894</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>40.90112204105026</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>45795</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="n">
-        <v>75.60177141592773</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>60.3004686782191</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>68.09769490471537</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>36.04348251398676</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>28.26395419963541</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>45802</v>
+        <v>45830</v>
       </c>
       <c r="B5" t="n">
-        <v>79.98771456203137</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>60.48982635881774</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>64.13615010036705</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>45.28276804316915</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>31.01285079601651</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>45809</v>
+        <v>45837</v>
       </c>
       <c r="B6" t="n">
-        <v>76.39394322837015</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>53.99607108358003</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>65.50358674052839</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>37.1265916488634</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>30.7767913676983</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>45816</v>
+        <v>45844</v>
       </c>
       <c r="B7" t="n">
-        <v>77.96419660027622</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>56.70432696718338</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>65.55440056678401</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>45.93542301871226</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>30.05654539738005</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>45823</v>
+        <v>45851</v>
       </c>
       <c r="B8" t="n">
-        <v>84.84307310122053</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>59.85446549032014</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>60.98064279056845</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>47.79297789503702</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>26.68009949202686</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>45830</v>
+        <v>45858</v>
       </c>
       <c r="B9" t="n">
-        <v>83.69337793727934</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>63.01982756731297</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>67.51450754019942</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>37.89658840824145</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>31.46724943099267</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>45837</v>
+        <v>45865</v>
       </c>
       <c r="B10" t="n">
-        <v>81.09561262051193</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>57.78918540156001</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>68.51671448203427</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>46.81688064622161</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>25.83026776930069</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>45844</v>
+        <v>45872</v>
       </c>
       <c r="B11" t="n">
-        <v>85.05512950108383</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>59.55148174040356</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>76.34135925100648</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>44.06390463468249</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>28.46449027892232</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>45851</v>
+        <v>45879</v>
       </c>
       <c r="B12" t="n">
-        <v>82.75706343863177</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>56.45701304515236</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>68.85446145036941</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>46.11030079997245</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>27.96050659299731</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>45858</v>
+        <v>45886</v>
       </c>
       <c r="B13" t="n">
-        <v>83.25553550568324</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>56.68576173897144</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>70.67312520459684</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>51.48396491326974</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>30.71965342029039</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>45865</v>
+        <v>45893</v>
       </c>
       <c r="B14" t="n">
-        <v>85.66189945912362</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>65.30892681898857</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>69.85320645383462</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>40.77305941998565</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>40.14098720787051</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>45872</v>
+        <v>45900</v>
       </c>
       <c r="B15" t="n">
-        <v>79.25304506172709</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>68.0720189378127</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>66.48922308427505</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>38.23131917821255</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>23.90348824924085</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>45879</v>
+        <v>45907</v>
       </c>
       <c r="B16" t="n">
-        <v>79.64772858367979</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>62.94725363132572</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>73.31012316435765</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>37.55242785187238</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>34.60778585953727</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>45886</v>
+        <v>45914</v>
       </c>
       <c r="B17" t="n">
-        <v>82.74052205986938</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>67.83766100333281</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>71.87405552978851</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>37.92094857517281</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>25.90207769171198</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>45893</v>
+        <v>45921</v>
       </c>
       <c r="B18" t="n">
-        <v>80.77508940817103</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>65.85830880607288</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>71.58215102057868</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>41.61449145292948</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>30.95540979174423</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>45900</v>
+        <v>45928</v>
       </c>
       <c r="B19" t="n">
-        <v>83.9331230545524</v>
+        <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>62.4195209815795</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>65.93209167346016</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>43.70575987408322</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>37.6891357212028</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>45907</v>
+        <v>45935</v>
       </c>
       <c r="B20" t="n">
-        <v>79.24618618263996</v>
+        <v>0</v>
       </c>
       <c r="C20" t="n">
-        <v>67.0338177161513</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>72.18855520561068</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>43.3834539966501</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>34.08064948814656</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>45914</v>
+        <v>45942</v>
       </c>
       <c r="B21" t="n">
-        <v>76.53176774196076</v>
+        <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>72.32861685409917</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>62.97356604226758</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>46.13591624518012</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>30.00274637847885</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>45921</v>
+        <v>45949</v>
       </c>
       <c r="B22" t="n">
-        <v>83.80080339517626</v>
+        <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>66.62140172591313</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>68.02980934034188</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>42.06500945938954</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>31.94270673158758</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>45928</v>
+        <v>45956</v>
       </c>
       <c r="B23" t="n">
-        <v>77.21915354170073</v>
+        <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>73.61151579972662</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>71.8356885062035</v>
+        <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>49.26767038578659</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>38.01250864279753</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>45935</v>
+        <v>45963</v>
       </c>
       <c r="B24" t="n">
-        <v>76.47198978736552</v>
+        <v>100</v>
       </c>
       <c r="C24" t="n">
-        <v>57.46219605422925</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>61.20799447347577</v>
+        <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>40.67671583381022</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>32.86284719862164</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>45942</v>
+        <v>45970</v>
       </c>
       <c r="B25" t="n">
-        <v>70.27304555305528</v>
+        <v>0</v>
       </c>
       <c r="C25" t="n">
-        <v>71.81702178220678</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>61.33263355232212</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>55.6008458329481</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>37.14034416224947</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>45949</v>
+        <v>45977</v>
       </c>
       <c r="B26" t="n">
-        <v>71.123094593673</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>69.46583533177622</v>
+        <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>62.13644927342862</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>45.12833673882503</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>36.94699324196819</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>45956</v>
+        <v>45984</v>
       </c>
       <c r="B27" t="n">
-        <v>71.25618136113874</v>
+        <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>68.5098529510777</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>59.10518209899083</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>37.71421221791859</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>34.64850057036104</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>45963</v>
+        <v>45991</v>
       </c>
       <c r="B28" t="n">
-        <v>65.62360567572395</v>
+        <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>70.66116075320083</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>54.73240064546218</v>
+        <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>36.64553750969444</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>46.32087439651698</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>45970</v>
+        <v>45998</v>
       </c>
       <c r="B29" t="n">
-        <v>68.37085128778847</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>62.93207728277289</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>58.36819374625238</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>44.41236207621593</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>40.7709702069191</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>45977</v>
+        <v>46005</v>
       </c>
       <c r="B30" t="n">
-        <v>63.65079381854794</v>
+        <v>0</v>
       </c>
       <c r="C30" t="n">
-        <v>70.59190068394406</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>53.78156211769125</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>40.88268607337075</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>30.62491984944801</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>45984</v>
+        <v>46012</v>
       </c>
       <c r="B31" t="n">
-        <v>62.85551357731842</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>73.48727381545875</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>57.24117384303771</v>
+        <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>45.57000247046046</v>
+        <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>39.96150353358752</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>45991</v>
+        <v>46019</v>
       </c>
       <c r="B32" t="n">
-        <v>60.29839772015148</v>
+        <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>78.55863500249548</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>51.97740566852503</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>44.36618812286773</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>37.05873649386762</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>45998</v>
+        <v>46026</v>
       </c>
       <c r="B33" t="n">
-        <v>66.15297746511523</v>
+        <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>71.16221324455248</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>58.38056515611156</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>41.63585543671564</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>43.60581177055744</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46005</v>
+        <v>46033</v>
       </c>
       <c r="B34" t="n">
-        <v>59.19082947981957</v>
+        <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>70.58955500019196</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>50.47112089234687</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>37.76603140965798</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>37.51619155607312</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46012</v>
+        <v>46040</v>
       </c>
       <c r="B35" t="n">
-        <v>54.85660880392871</v>
+        <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>72.4047365315442</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>51.05364317858058</v>
+        <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>34.42576387657068</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>40.71752482236769</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46019</v>
+        <v>46047</v>
       </c>
       <c r="B36" t="n">
-        <v>59.47725367954299</v>
+        <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>78.66160847080829</v>
+        <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>53.78029761426463</v>
+        <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>39.7674252396649</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>43.68661578258849</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46026</v>
+        <v>46054</v>
       </c>
       <c r="B37" t="n">
-        <v>52.52388628091263</v>
+        <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>76.90323973275639</v>
+        <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>47.0983518712486</v>
+        <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>46.28199397161736</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>45.61988352177853</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46033</v>
+        <v>46061</v>
       </c>
       <c r="B38" t="n">
-        <v>56.19920613742198</v>
+        <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>74.05742977316713</v>
+        <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>51.0641233720842</v>
+        <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>43.07046872065102</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>37.8458731953063</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46040</v>
+        <v>46068</v>
       </c>
       <c r="B39" t="n">
-        <v>49.29850754714179</v>
+        <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>78.81777561480637</v>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>54.03977354203469</v>
+        <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>35.77130610644006</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>41.799249958597</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46047</v>
+        <v>46075</v>
       </c>
       <c r="B40" t="n">
-        <v>51.02255605760422</v>
+        <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>77.74125137386275</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>45.18229309918266</v>
+        <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>42.86590462925591</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>41.72766973574833</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B41" t="n">
-        <v>55.65457106318186</v>
+        <v>0</v>
       </c>
       <c r="C41" t="n">
-        <v>81.81575643271979</v>
+        <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>50.59655981264656</v>
+        <v>0</v>
       </c>
       <c r="E41" t="n">
-        <v>43.92658689864418</v>
+        <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>41.50433012852868</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46061</v>
+        <v>46089</v>
       </c>
       <c r="B42" t="n">
-        <v>57.56267497359222</v>
+        <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>75.72119938919647</v>
+        <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>51.01116520514926</v>
+        <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>37.58071281899434</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>51.66966009837929</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46068</v>
+        <v>46096</v>
       </c>
       <c r="B43" t="n">
-        <v>56.36678832650075</v>
+        <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>77.80699847243247</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>52.91392427061916</v>
+        <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>42.76862552972764</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>46.71796605953009</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46075</v>
+        <v>46103</v>
       </c>
       <c r="B44" t="n">
-        <v>56.22560578250934</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>78.13744974041255</v>
+        <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>47.33751495381513</v>
+        <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>42.29104359223</v>
+        <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>40.54469947677747</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>46082</v>
+        <v>46110</v>
       </c>
       <c r="B45" t="n">
-        <v>56.59265313491534</v>
+        <v>0</v>
       </c>
       <c r="C45" t="n">
-        <v>74.44005785453035</v>
+        <v>0</v>
       </c>
       <c r="D45" t="n">
-        <v>47.70260630853597</v>
+        <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>36.28514851084688</v>
+        <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>49.74987916076812</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>46089</v>
+        <v>46117</v>
       </c>
       <c r="B46" t="n">
-        <v>54.1733602790771</v>
+        <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>82.06683404943477</v>
+        <v>0</v>
       </c>
       <c r="D46" t="n">
-        <v>53.97177553030362</v>
+        <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>43.78893680174141</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>55.05725223903092</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>46096</v>
+        <v>46124</v>
       </c>
       <c r="B47" t="n">
-        <v>57.73503272011752</v>
+        <v>0</v>
       </c>
       <c r="C47" t="n">
-        <v>82.51480932401367</v>
+        <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>54.15399758323399</v>
+        <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>44.80392263184117</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>51.18868457161636</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>46103</v>
+        <v>46131</v>
       </c>
       <c r="B48" t="n">
-        <v>59.95147621599687</v>
+        <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>82.07927735598162</v>
+        <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>54.97374023695512</v>
+        <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>47.41525621587638</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>41.47153974402708</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>46110</v>
+        <v>46138</v>
       </c>
       <c r="B49" t="n">
-        <v>66.07496332611659</v>
+        <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>81.70871029002883</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>56.30840906013082</v>
+        <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>47.26901026017451</v>
+        <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>46.10227939480951</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>46117</v>
+        <v>46145</v>
       </c>
       <c r="B50" t="n">
-        <v>65.61222987589809</v>
+        <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>77.5738111494454</v>
+        <v>0</v>
       </c>
       <c r="D50" t="n">
-        <v>54.347509173393</v>
+        <v>0</v>
       </c>
       <c r="E50" t="n">
-        <v>35.11165316021454</v>
+        <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>53.59705636145237</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>46124</v>
+        <v>46152</v>
       </c>
       <c r="B51" t="n">
-        <v>61.05217373228614</v>
+        <v>0</v>
       </c>
       <c r="C51" t="n">
-        <v>82.14094812070327</v>
+        <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>58.25762389039924</v>
+        <v>0</v>
       </c>
       <c r="E51" t="n">
-        <v>37.31087480042439</v>
+        <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>46.18892998066213</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>46131</v>
+        <v>46159</v>
       </c>
       <c r="B52" t="n">
-        <v>69.12892754821368</v>
+        <v>17</v>
       </c>
       <c r="C52" t="n">
-        <v>83.04090663977527</v>
+        <v>0</v>
       </c>
       <c r="D52" t="n">
-        <v>59.6503345132489</v>
+        <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>44.5751763360433</v>
+        <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>51.28508163415354</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>46138</v>
+        <v>46166</v>
       </c>
       <c r="B53" t="n">
-        <v>68.84475315875105</v>
+        <v>28</v>
       </c>
       <c r="C53" t="n">
-        <v>81.79089092311352</v>
+        <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>57.8569457459209</v>
+        <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>44.56892975456105</v>
+        <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>53.09853621371735</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B54" t="n">
+        <v>21</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1517,51 +1542,51 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vitrificação automotiva</t>
+          <t>polimento automotivo</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69.84377184491193</v>
+        <v>3.132075471698113</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>polimento automotivo</t>
+          <t>ppf automotivo</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>69.34607537074066</v>
+        <v>0.3018867924528302</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>higienização automotiva</t>
+          <t>vitrificação automotiva</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60.04295311198792</v>
+        <v>0.1509433962264151</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>lavagem técnica carro</t>
+          <t>higienização automotiva</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>42.59958634037896</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ppf automotivo</t>
+          <t>lavagem técnica carro</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>38.14349273757428</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1592,7 +1617,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>39.53985435118781</v>
+        <v>59.25925925925925</v>
       </c>
     </row>
     <row r="3">
@@ -1602,27 +1627,27 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>22.2051772444626</v>
+        <v>29.62962962962963</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>lavagem técnica carro</t>
+          <t>higienização automotiva</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-4.661613827872214</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>higienização automotiva</t>
+          <t>lavagem técnica carro</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-20.14582131127154</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1632,7 +1657,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-24.2263510302619</v>
+        <v>-36.44444444444444</v>
       </c>
     </row>
   </sheetData>
@@ -2592,7 +2617,7 @@
         <v>2022</v>
       </c>
       <c r="D67" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -3558,7 +3583,7 @@
         <v>2023</v>
       </c>
       <c r="D136" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
@@ -5308,7 +5333,7 @@
         <v>2026</v>
       </c>
       <c r="D261" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="262">
@@ -5322,7 +5347,7 @@
         <v>2026</v>
       </c>
       <c r="D262" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
     </row>
     <row r="263">
@@ -5407,7 +5432,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.5217391304347826</v>
+        <v>4.347826086956522</v>
       </c>
     </row>
     <row r="7">
@@ -5437,7 +5462,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.272727272727273</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -5477,7 +5502,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4.545454545454546</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5519,7 +5544,7 @@
         <v>2022</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9615384615384616</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -5527,7 +5552,7 @@
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>1.886792452830189</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -5551,7 +5576,7 @@
         <v>2026</v>
       </c>
       <c r="B7" t="n">
-        <v>0.5454545454545454</v>
+        <v>4.545454545454546</v>
       </c>
     </row>
   </sheetData>
@@ -5565,7 +5590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5580,86 +5605,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Uberaba</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Contagem</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Juiz de Fora</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Uberlândia</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Santa Luzia</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Belo Horizonte</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Betim</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Montes Claros</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>57</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>